<commit_message>
GUI sprints of 3 weeks, new version numbering
Former-commit-id: 11127a37e8d8f2314bd40ce6faea5b8d768499f8
Former-commit-id: 7a61868a3bf39c6b6fd739f9f572ceaa7d591152
</commit_message>
<xml_diff>
--- a/documents/planning/BOOT-SprintGoals  Releases 2017.xlsx
+++ b/documents/planning/BOOT-SprintGoals  Releases 2017.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="148">
   <si>
     <t>D-Hydro team (BOOT)</t>
   </si>
@@ -437,6 +437,30 @@
   </si>
   <si>
     <t>D-FlowFM: Editor voor General structure (M), Visualisatie Grid snapped features (S), Observationpoints en mappenstructuur</t>
+  </si>
+  <si>
+    <t>Do 25 mei: Rehearsal release D-Hydro 1.3.0 / SOBEK 3.7.0</t>
+  </si>
+  <si>
+    <t>Do 22 juni: Release 2017.1 D-Hydro 1.3.1 / SOBEK 3.7.1</t>
+  </si>
+  <si>
+    <t>Patch release NGHS D-Hydro 1.3.2 / SOBEK 3.7.2</t>
+  </si>
+  <si>
+    <t>Patch release D-Hydro 1.3.3 / SOBEK 3.7.3</t>
+  </si>
+  <si>
+    <t>Patch release D-Hydro 1.3.4 / SOBEK 3.7.4</t>
+  </si>
+  <si>
+    <t>Do 12 okt: Rehearsal release D-Hydro 1.3.5 / SOBEK 3.7.5</t>
+  </si>
+  <si>
+    <t>Do 9 nov: Release 2017.2 D-Hydro 1.3.6 / SOBEK 3.7.6</t>
+  </si>
+  <si>
+    <t>Patch release D-Hydro 1.3.7 / SOBEK 3.7.7</t>
   </si>
 </sst>
 </file>
@@ -542,7 +566,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -639,6 +663,15 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -646,7 +679,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -764,11 +797,60 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="1" fillId="4" borderId="10" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="16" fontId="1" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="1" fillId="4" borderId="0" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="1" fillId="3" borderId="10" xfId="2" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="10" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1502,24 +1584,24 @@
       </c>
     </row>
     <row r="20" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="5" t="s">
+      <c r="A20" s="47" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="47" t="s">
         <v>26</v>
       </c>
-      <c r="C20" s="6">
+      <c r="C20" s="48">
         <v>42877</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="49" t="s">
         <v>128</v>
       </c>
-      <c r="E20" s="17">
+      <c r="E20" s="50">
         <v>0.8</v>
       </c>
       <c r="F20" s="17"/>
       <c r="G20" s="7" t="s">
-        <v>91</v>
+        <v>140</v>
       </c>
       <c r="H20" s="38" t="s">
         <v>122</v>
@@ -1532,15 +1614,15 @@
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A21" s="41"/>
-      <c r="B21" s="41" t="s">
+      <c r="A21" s="23"/>
+      <c r="B21" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="C21" s="42">
+      <c r="C21" s="51">
         <v>42884</v>
       </c>
-      <c r="D21" s="43"/>
-      <c r="E21" s="43"/>
+      <c r="D21" s="44"/>
+      <c r="E21" s="44"/>
       <c r="F21" s="16"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3" t="s">
@@ -1550,19 +1632,17 @@
       <c r="J21" s="3"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B22" s="3" t="s">
+      <c r="A22" s="23"/>
+      <c r="B22" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="C22" s="4">
+      <c r="C22" s="51">
         <v>42891</v>
       </c>
-      <c r="D22" s="22" t="s">
+      <c r="D22" s="52" t="s">
         <v>128</v>
       </c>
-      <c r="E22" s="16">
+      <c r="E22" s="44">
         <v>0.8</v>
       </c>
       <c r="F22" s="16"/>
@@ -1574,15 +1654,17 @@
       <c r="J22" s="3"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" s="41"/>
-      <c r="B23" s="41" t="s">
+      <c r="A23" s="53" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23" s="53" t="s">
         <v>30</v>
       </c>
-      <c r="C23" s="42">
+      <c r="C23" s="54">
         <v>42898</v>
       </c>
-      <c r="D23" s="43"/>
-      <c r="E23" s="45"/>
+      <c r="D23" s="55"/>
+      <c r="E23" s="56"/>
       <c r="F23" s="18"/>
       <c r="G23" s="3"/>
       <c r="H23" s="3" t="s">
@@ -1596,24 +1678,22 @@
       </c>
     </row>
     <row r="24" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A24" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="B24" s="8" t="s">
+      <c r="A24" s="11"/>
+      <c r="B24" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="C24" s="9">
+      <c r="C24" s="57">
         <v>42905</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="D24" s="11" t="s">
         <v>138</v>
       </c>
-      <c r="E24" s="19">
+      <c r="E24" s="20">
         <v>1</v>
       </c>
       <c r="F24" s="19"/>
       <c r="G24" s="10" t="s">
-        <v>97</v>
+        <v>141</v>
       </c>
       <c r="H24" s="3" t="s">
         <v>116</v>
@@ -1624,15 +1704,15 @@
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A25" s="41"/>
-      <c r="B25" s="41" t="s">
+      <c r="A25" s="23"/>
+      <c r="B25" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="C25" s="42">
+      <c r="C25" s="51">
         <v>42912</v>
       </c>
-      <c r="D25" s="43"/>
-      <c r="E25" s="43"/>
+      <c r="D25" s="44"/>
+      <c r="E25" s="44"/>
       <c r="F25" s="16"/>
       <c r="G25" s="3"/>
       <c r="H25" s="38" t="s">
@@ -1642,19 +1722,19 @@
       <c r="J25" s="3"/>
     </row>
     <row r="26" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B26" s="3" t="s">
+      <c r="A26" s="53" t="s">
+        <v>31</v>
+      </c>
+      <c r="B26" s="53" t="s">
         <v>35</v>
       </c>
-      <c r="C26" s="4">
+      <c r="C26" s="54">
         <v>42919</v>
       </c>
-      <c r="D26" s="16" t="s">
+      <c r="D26" s="55" t="s">
         <v>139</v>
       </c>
-      <c r="E26" s="16">
+      <c r="E26" s="55">
         <v>1</v>
       </c>
       <c r="F26" s="16"/>
@@ -1663,19 +1743,19 @@
       <c r="I26" s="3"/>
       <c r="J26" s="3"/>
     </row>
-    <row r="27" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A27" s="41"/>
-      <c r="B27" s="41" t="s">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" s="23"/>
+      <c r="B27" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="C27" s="42">
+      <c r="C27" s="51">
         <v>42926</v>
       </c>
-      <c r="D27" s="43"/>
-      <c r="E27" s="43"/>
+      <c r="D27" s="44"/>
+      <c r="E27" s="44"/>
       <c r="F27" s="16"/>
       <c r="G27" s="3" t="s">
-        <v>92</v>
+        <v>142</v>
       </c>
       <c r="H27" s="3" t="s">
         <v>132</v>
@@ -1686,19 +1766,17 @@
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B28" s="3" t="s">
+      <c r="A28" s="23"/>
+      <c r="B28" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="C28" s="4">
+      <c r="C28" s="51">
         <v>42933</v>
       </c>
-      <c r="D28" s="16" t="s">
+      <c r="D28" s="44" t="s">
         <v>81</v>
       </c>
-      <c r="E28" s="16">
+      <c r="E28" s="44">
         <v>1</v>
       </c>
       <c r="F28" s="16"/>
@@ -1710,15 +1788,17 @@
       <c r="J28" s="3"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A29" s="41"/>
-      <c r="B29" s="41" t="s">
+      <c r="A29" s="53" t="s">
+        <v>34</v>
+      </c>
+      <c r="B29" s="53" t="s">
         <v>39</v>
       </c>
-      <c r="C29" s="42">
+      <c r="C29" s="54">
         <v>42940</v>
       </c>
-      <c r="D29" s="43"/>
-      <c r="E29" s="43"/>
+      <c r="D29" s="55"/>
+      <c r="E29" s="55"/>
       <c r="F29" s="16"/>
       <c r="G29" s="3"/>
       <c r="H29" s="38" t="s">
@@ -1728,19 +1808,17 @@
       <c r="J29" s="3"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B30" s="3" t="s">
+      <c r="A30" s="23"/>
+      <c r="B30" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="C30" s="4">
+      <c r="C30" s="51">
         <v>42947</v>
       </c>
-      <c r="D30" s="21" t="s">
+      <c r="D30" s="58" t="s">
         <v>81</v>
       </c>
-      <c r="E30" s="16">
+      <c r="E30" s="44">
         <v>1</v>
       </c>
       <c r="F30" s="16"/>
@@ -1750,18 +1828,18 @@
       <c r="J30" s="3"/>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A31" s="41"/>
-      <c r="B31" s="41" t="s">
+      <c r="A31" s="23"/>
+      <c r="B31" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="C31" s="42">
+      <c r="C31" s="51">
         <v>42954</v>
       </c>
-      <c r="D31" s="43"/>
-      <c r="E31" s="43"/>
+      <c r="D31" s="44"/>
+      <c r="E31" s="44"/>
       <c r="F31" s="16"/>
       <c r="G31" s="3" t="s">
-        <v>93</v>
+        <v>143</v>
       </c>
       <c r="H31" s="3" t="s">
         <v>133</v>
@@ -1772,19 +1850,19 @@
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A32" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B32" s="3" t="s">
+      <c r="A32" s="53" t="s">
+        <v>37</v>
+      </c>
+      <c r="B32" s="53" t="s">
         <v>44</v>
       </c>
-      <c r="C32" s="4">
+      <c r="C32" s="54">
         <v>42961</v>
       </c>
-      <c r="D32" s="16" t="s">
+      <c r="D32" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="E32" s="16">
+      <c r="E32" s="55">
         <v>1</v>
       </c>
       <c r="F32" s="16"/>
@@ -1796,15 +1874,15 @@
       <c r="J32" s="3"/>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A33" s="41"/>
-      <c r="B33" s="41" t="s">
+      <c r="A33" s="23"/>
+      <c r="B33" s="23" t="s">
         <v>45</v>
       </c>
-      <c r="C33" s="42">
+      <c r="C33" s="51">
         <v>42968</v>
       </c>
-      <c r="D33" s="43"/>
-      <c r="E33" s="43"/>
+      <c r="D33" s="44"/>
+      <c r="E33" s="44"/>
       <c r="F33" s="16"/>
       <c r="G33" s="3"/>
       <c r="H33" s="38" t="s">
@@ -1814,19 +1892,17 @@
       <c r="J33" s="3"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A34" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B34" s="3" t="s">
+      <c r="A34" s="23"/>
+      <c r="B34" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="C34" s="4">
+      <c r="C34" s="51">
         <v>42975</v>
       </c>
-      <c r="D34" s="16" t="s">
+      <c r="D34" s="44" t="s">
         <v>82</v>
       </c>
-      <c r="E34" s="16">
+      <c r="E34" s="44">
         <v>1</v>
       </c>
       <c r="F34" s="16"/>
@@ -1836,20 +1912,22 @@
       <c r="J34" s="3"/>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A35" s="41"/>
-      <c r="B35" s="41" t="s">
+      <c r="A35" s="53" t="s">
+        <v>40</v>
+      </c>
+      <c r="B35" s="53" t="s">
         <v>48</v>
       </c>
-      <c r="C35" s="42">
+      <c r="C35" s="54">
         <v>42982</v>
       </c>
-      <c r="D35" s="43"/>
-      <c r="E35" s="43" t="s">
+      <c r="D35" s="55"/>
+      <c r="E35" s="55" t="s">
         <v>103</v>
       </c>
       <c r="F35" s="16"/>
       <c r="G35" s="3" t="s">
-        <v>94</v>
+        <v>144</v>
       </c>
       <c r="H35" s="3"/>
       <c r="I35" s="3"/>
@@ -1858,19 +1936,17 @@
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A36" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B36" s="3" t="s">
+      <c r="A36" s="23"/>
+      <c r="B36" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="C36" s="4">
+      <c r="C36" s="51">
         <v>42989</v>
       </c>
-      <c r="D36" s="16" t="s">
+      <c r="D36" s="44" t="s">
         <v>82</v>
       </c>
-      <c r="E36" s="16">
+      <c r="E36" s="44">
         <v>1</v>
       </c>
       <c r="F36" s="16"/>
@@ -1882,15 +1958,15 @@
       <c r="J36" s="3"/>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A37" s="41"/>
-      <c r="B37" s="41" t="s">
+      <c r="A37" s="23"/>
+      <c r="B37" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="C37" s="42">
+      <c r="C37" s="51">
         <v>42996</v>
       </c>
-      <c r="D37" s="43"/>
-      <c r="E37" s="43"/>
+      <c r="D37" s="44"/>
+      <c r="E37" s="44"/>
       <c r="F37" s="16"/>
       <c r="G37" s="3"/>
       <c r="H37" s="3" t="s">
@@ -1900,19 +1976,19 @@
       <c r="J37" s="3"/>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A38" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B38" s="3" t="s">
+      <c r="A38" s="53" t="s">
+        <v>43</v>
+      </c>
+      <c r="B38" s="53" t="s">
         <v>53</v>
       </c>
-      <c r="C38" s="4">
+      <c r="C38" s="54">
         <v>43003</v>
       </c>
-      <c r="D38" s="16" t="s">
+      <c r="D38" s="55" t="s">
         <v>87</v>
       </c>
-      <c r="E38" s="16">
+      <c r="E38" s="55">
         <v>1</v>
       </c>
       <c r="F38" s="16"/>
@@ -1924,15 +2000,15 @@
       <c r="J38" s="3"/>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A39" s="41"/>
-      <c r="B39" s="41" t="s">
+      <c r="A39" s="23"/>
+      <c r="B39" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="C39" s="42">
+      <c r="C39" s="51">
         <v>43010</v>
       </c>
-      <c r="D39" s="43"/>
-      <c r="E39" s="43"/>
+      <c r="D39" s="44"/>
+      <c r="E39" s="44"/>
       <c r="F39" s="16"/>
       <c r="G39" s="3"/>
       <c r="H39" s="3"/>
@@ -1942,24 +2018,22 @@
       </c>
     </row>
     <row r="40" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A40" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="B40" s="5" t="s">
+      <c r="A40" s="59"/>
+      <c r="B40" s="59" t="s">
         <v>56</v>
       </c>
-      <c r="C40" s="6">
+      <c r="C40" s="60">
         <v>43017</v>
       </c>
-      <c r="D40" s="5" t="s">
+      <c r="D40" s="59" t="s">
         <v>104</v>
       </c>
-      <c r="E40" s="17">
+      <c r="E40" s="61">
         <v>1</v>
       </c>
       <c r="F40" s="17"/>
       <c r="G40" s="7" t="s">
-        <v>95</v>
+        <v>145</v>
       </c>
       <c r="H40" s="38" t="s">
         <v>135</v>
@@ -1970,15 +2044,17 @@
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A41" s="41"/>
-      <c r="B41" s="41" t="s">
+      <c r="A41" s="53" t="s">
+        <v>46</v>
+      </c>
+      <c r="B41" s="53" t="s">
         <v>58</v>
       </c>
-      <c r="C41" s="42">
+      <c r="C41" s="54">
         <v>43024</v>
       </c>
-      <c r="D41" s="43"/>
-      <c r="E41" s="43"/>
+      <c r="D41" s="55"/>
+      <c r="E41" s="55"/>
       <c r="F41" s="16"/>
       <c r="G41" s="3"/>
       <c r="H41" s="3" t="s">
@@ -1988,19 +2064,17 @@
       <c r="J41" s="3"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A42" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="B42" s="3" t="s">
+      <c r="A42" s="23"/>
+      <c r="B42" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="C42" s="4">
+      <c r="C42" s="51">
         <v>43031</v>
       </c>
-      <c r="D42" s="21" t="s">
+      <c r="D42" s="58" t="s">
         <v>86</v>
       </c>
-      <c r="E42" s="16">
+      <c r="E42" s="44">
         <v>0.8</v>
       </c>
       <c r="F42" s="16"/>
@@ -2014,15 +2088,15 @@
       <c r="J42" s="3"/>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A43" s="3"/>
-      <c r="B43" s="3" t="s">
+      <c r="A43" s="23"/>
+      <c r="B43" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="C43" s="4">
+      <c r="C43" s="51">
         <v>43038</v>
       </c>
-      <c r="D43" s="16"/>
-      <c r="E43" s="16"/>
+      <c r="D43" s="44"/>
+      <c r="E43" s="44"/>
       <c r="F43" s="16"/>
       <c r="G43" s="3"/>
       <c r="H43" s="3"/>
@@ -2034,24 +2108,24 @@
       </c>
     </row>
     <row r="44" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A44" s="8" t="s">
+      <c r="A44" s="62" t="s">
         <v>60</v>
       </c>
-      <c r="B44" s="8" t="s">
+      <c r="B44" s="62" t="s">
         <v>62</v>
       </c>
-      <c r="C44" s="9">
+      <c r="C44" s="63">
         <v>43045</v>
       </c>
-      <c r="D44" s="8" t="s">
+      <c r="D44" s="62" t="s">
         <v>129</v>
       </c>
-      <c r="E44" s="20">
+      <c r="E44" s="64">
         <v>1</v>
       </c>
       <c r="F44" s="20"/>
       <c r="G44" s="12" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="H44" s="40"/>
       <c r="I44" s="11"/>
@@ -2060,15 +2134,15 @@
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A45" s="3"/>
-      <c r="B45" s="3" t="s">
+      <c r="A45" s="23"/>
+      <c r="B45" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="C45" s="4">
+      <c r="C45" s="51">
         <v>43052</v>
       </c>
-      <c r="D45" s="16"/>
-      <c r="E45" s="16"/>
+      <c r="D45" s="44"/>
+      <c r="E45" s="44"/>
       <c r="F45" s="16"/>
       <c r="G45" s="3"/>
       <c r="H45" s="3" t="s">
@@ -2078,19 +2152,17 @@
       <c r="J45" s="3"/>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A46" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="B46" s="3" t="s">
+      <c r="A46" s="23"/>
+      <c r="B46" s="23" t="s">
         <v>65</v>
       </c>
-      <c r="C46" s="4">
+      <c r="C46" s="51">
         <v>43059</v>
       </c>
-      <c r="D46" s="16" t="s">
+      <c r="D46" s="44" t="s">
         <v>83</v>
       </c>
-      <c r="E46" s="16">
+      <c r="E46" s="44">
         <v>1</v>
       </c>
       <c r="F46" s="16"/>
@@ -2102,15 +2174,17 @@
       <c r="J46" s="3"/>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A47" s="3"/>
-      <c r="B47" s="3" t="s">
+      <c r="A47" s="53" t="s">
+        <v>63</v>
+      </c>
+      <c r="B47" s="53" t="s">
         <v>66</v>
       </c>
-      <c r="C47" s="4">
+      <c r="C47" s="54">
         <v>43066</v>
       </c>
-      <c r="D47" s="16"/>
-      <c r="E47" s="16"/>
+      <c r="D47" s="55"/>
+      <c r="E47" s="55"/>
       <c r="F47" s="16"/>
       <c r="G47" s="3"/>
       <c r="H47" s="38" t="s">
@@ -2120,17 +2194,15 @@
       <c r="J47" s="3"/>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A48" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="B48" s="3" t="s">
+      <c r="A48" s="23"/>
+      <c r="B48" s="23" t="s">
         <v>67</v>
       </c>
-      <c r="C48" s="4">
+      <c r="C48" s="51">
         <v>43073</v>
       </c>
-      <c r="D48" s="16"/>
-      <c r="E48" s="16">
+      <c r="D48" s="44"/>
+      <c r="E48" s="44">
         <v>1</v>
       </c>
       <c r="F48" s="16"/>
@@ -2142,18 +2214,18 @@
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A49" s="3"/>
-      <c r="B49" s="3" t="s">
+      <c r="A49" s="23"/>
+      <c r="B49" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="C49" s="4">
+      <c r="C49" s="51">
         <v>43080</v>
       </c>
-      <c r="D49" s="16"/>
-      <c r="E49" s="16"/>
+      <c r="D49" s="44"/>
+      <c r="E49" s="44"/>
       <c r="F49" s="16"/>
       <c r="G49" s="3" t="s">
-        <v>96</v>
+        <v>147</v>
       </c>
       <c r="H49" s="3"/>
       <c r="I49" s="3"/>
@@ -2189,7 +2261,7 @@
       </c>
       <c r="B52" s="27"/>
       <c r="C52" s="27"/>
-      <c r="D52" s="46" t="s">
+      <c r="D52" s="45" t="s">
         <v>83</v>
       </c>
       <c r="E52" s="28"/>
@@ -2203,7 +2275,7 @@
       <c r="A53" s="30"/>
       <c r="B53" s="23"/>
       <c r="C53" s="23"/>
-      <c r="D53" s="47" t="s">
+      <c r="D53" s="46" t="s">
         <v>129</v>
       </c>
       <c r="E53" s="24"/>
@@ -2217,7 +2289,7 @@
       <c r="A54" s="30"/>
       <c r="B54" s="23"/>
       <c r="C54" s="23"/>
-      <c r="D54" s="47" t="s">
+      <c r="D54" s="46" t="s">
         <v>84</v>
       </c>
       <c r="E54" s="23"/>
@@ -2231,7 +2303,7 @@
       <c r="A55" s="30"/>
       <c r="B55" s="23"/>
       <c r="C55" s="23"/>
-      <c r="D55" s="47" t="s">
+      <c r="D55" s="46" t="s">
         <v>102</v>
       </c>
       <c r="E55" s="23"/>

</xml_diff>

<commit_message>
Merged revision(s) 37408-37412 from trunk/delta-shell/Products/NGHS: SOBEK3-1004 Fixed integration tests after they broke :( ........ GUI sprints of 3 weeks, new version numbering ........ Sequential sprint numbering ........ Fix failing SOBEK import and Compare tests Default value for Iadvec1D has been changed (from 1 to 2) ........
Former-commit-id: 9f20c852a3303589f813165e3092846377e70678
Former-commit-id: 78869cf7e09987b014f1a2b12ef9bd18f71961d3
</commit_message>
<xml_diff>
--- a/documents/planning/BOOT-SprintGoals  Releases 2017.xlsx
+++ b/documents/planning/BOOT-SprintGoals  Releases 2017.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="148">
   <si>
     <t>D-Hydro team (BOOT)</t>
   </si>
@@ -437,6 +437,30 @@
   </si>
   <si>
     <t>D-FlowFM: Editor voor General structure (M), Visualisatie Grid snapped features (S), Observationpoints en mappenstructuur</t>
+  </si>
+  <si>
+    <t>Do 25 mei: Rehearsal release D-Hydro 1.3.0 / SOBEK 3.7.0</t>
+  </si>
+  <si>
+    <t>Do 22 juni: Release 2017.1 D-Hydro 1.3.1 / SOBEK 3.7.1</t>
+  </si>
+  <si>
+    <t>Patch release NGHS D-Hydro 1.3.2 / SOBEK 3.7.2</t>
+  </si>
+  <si>
+    <t>Patch release D-Hydro 1.3.3 / SOBEK 3.7.3</t>
+  </si>
+  <si>
+    <t>Patch release D-Hydro 1.3.4 / SOBEK 3.7.4</t>
+  </si>
+  <si>
+    <t>Do 12 okt: Rehearsal release D-Hydro 1.3.5 / SOBEK 3.7.5</t>
+  </si>
+  <si>
+    <t>Do 9 nov: Release 2017.2 D-Hydro 1.3.6 / SOBEK 3.7.6</t>
+  </si>
+  <si>
+    <t>Patch release D-Hydro 1.3.7 / SOBEK 3.7.7</t>
   </si>
 </sst>
 </file>
@@ -542,7 +566,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -639,6 +663,15 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -646,7 +679,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -764,11 +797,63 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="1" fillId="4" borderId="10" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="16" fontId="1" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="1" fillId="4" borderId="0" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="1" fillId="3" borderId="10" xfId="2" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="10" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1502,24 +1587,24 @@
       </c>
     </row>
     <row r="20" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="5" t="s">
+      <c r="A20" s="47" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="47" t="s">
         <v>26</v>
       </c>
-      <c r="C20" s="6">
+      <c r="C20" s="48">
         <v>42877</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="49" t="s">
         <v>128</v>
       </c>
-      <c r="E20" s="17">
+      <c r="E20" s="50">
         <v>0.8</v>
       </c>
       <c r="F20" s="17"/>
       <c r="G20" s="7" t="s">
-        <v>91</v>
+        <v>140</v>
       </c>
       <c r="H20" s="38" t="s">
         <v>122</v>
@@ -1532,15 +1617,15 @@
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A21" s="41"/>
-      <c r="B21" s="41" t="s">
+      <c r="A21" s="23"/>
+      <c r="B21" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="C21" s="42">
+      <c r="C21" s="51">
         <v>42884</v>
       </c>
-      <c r="D21" s="43"/>
-      <c r="E21" s="43"/>
+      <c r="D21" s="44"/>
+      <c r="E21" s="44"/>
       <c r="F21" s="16"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3" t="s">
@@ -1550,19 +1635,17 @@
       <c r="J21" s="3"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B22" s="3" t="s">
+      <c r="A22" s="23"/>
+      <c r="B22" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="C22" s="4">
+      <c r="C22" s="51">
         <v>42891</v>
       </c>
-      <c r="D22" s="22" t="s">
+      <c r="D22" s="52" t="s">
         <v>128</v>
       </c>
-      <c r="E22" s="16">
+      <c r="E22" s="44">
         <v>0.8</v>
       </c>
       <c r="F22" s="16"/>
@@ -1574,15 +1657,17 @@
       <c r="J22" s="3"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" s="41"/>
-      <c r="B23" s="41" t="s">
+      <c r="A23" s="53" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23" s="53" t="s">
         <v>30</v>
       </c>
-      <c r="C23" s="42">
+      <c r="C23" s="54">
         <v>42898</v>
       </c>
-      <c r="D23" s="43"/>
-      <c r="E23" s="45"/>
+      <c r="D23" s="55"/>
+      <c r="E23" s="56"/>
       <c r="F23" s="18"/>
       <c r="G23" s="3"/>
       <c r="H23" s="3" t="s">
@@ -1596,24 +1681,22 @@
       </c>
     </row>
     <row r="24" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A24" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="B24" s="8" t="s">
+      <c r="A24" s="11"/>
+      <c r="B24" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="C24" s="9">
+      <c r="C24" s="57">
         <v>42905</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="D24" s="11" t="s">
         <v>138</v>
       </c>
-      <c r="E24" s="19">
+      <c r="E24" s="20">
         <v>1</v>
       </c>
       <c r="F24" s="19"/>
       <c r="G24" s="10" t="s">
-        <v>97</v>
+        <v>141</v>
       </c>
       <c r="H24" s="3" t="s">
         <v>116</v>
@@ -1624,15 +1707,15 @@
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A25" s="41"/>
-      <c r="B25" s="41" t="s">
+      <c r="A25" s="23"/>
+      <c r="B25" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="C25" s="42">
+      <c r="C25" s="51">
         <v>42912</v>
       </c>
-      <c r="D25" s="43"/>
-      <c r="E25" s="43"/>
+      <c r="D25" s="44"/>
+      <c r="E25" s="44"/>
       <c r="F25" s="16"/>
       <c r="G25" s="3"/>
       <c r="H25" s="38" t="s">
@@ -1642,19 +1725,19 @@
       <c r="J25" s="3"/>
     </row>
     <row r="26" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B26" s="3" t="s">
+      <c r="A26" s="53" t="s">
+        <v>31</v>
+      </c>
+      <c r="B26" s="53" t="s">
         <v>35</v>
       </c>
-      <c r="C26" s="4">
+      <c r="C26" s="54">
         <v>42919</v>
       </c>
-      <c r="D26" s="16" t="s">
+      <c r="D26" s="55" t="s">
         <v>139</v>
       </c>
-      <c r="E26" s="16">
+      <c r="E26" s="55">
         <v>1</v>
       </c>
       <c r="F26" s="16"/>
@@ -1663,19 +1746,19 @@
       <c r="I26" s="3"/>
       <c r="J26" s="3"/>
     </row>
-    <row r="27" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A27" s="41"/>
-      <c r="B27" s="41" t="s">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" s="23"/>
+      <c r="B27" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="C27" s="42">
+      <c r="C27" s="51">
         <v>42926</v>
       </c>
-      <c r="D27" s="43"/>
-      <c r="E27" s="43"/>
+      <c r="D27" s="44"/>
+      <c r="E27" s="44"/>
       <c r="F27" s="16"/>
       <c r="G27" s="3" t="s">
-        <v>92</v>
+        <v>142</v>
       </c>
       <c r="H27" s="3" t="s">
         <v>132</v>
@@ -1686,19 +1769,17 @@
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B28" s="3" t="s">
+      <c r="A28" s="23"/>
+      <c r="B28" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="C28" s="4">
+      <c r="C28" s="51">
         <v>42933</v>
       </c>
-      <c r="D28" s="16" t="s">
+      <c r="D28" s="44" t="s">
         <v>81</v>
       </c>
-      <c r="E28" s="16">
+      <c r="E28" s="44">
         <v>1</v>
       </c>
       <c r="F28" s="16"/>
@@ -1710,15 +1791,17 @@
       <c r="J28" s="3"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A29" s="41"/>
-      <c r="B29" s="41" t="s">
+      <c r="A29" s="53" t="s">
+        <v>34</v>
+      </c>
+      <c r="B29" s="53" t="s">
         <v>39</v>
       </c>
-      <c r="C29" s="42">
+      <c r="C29" s="54">
         <v>42940</v>
       </c>
-      <c r="D29" s="43"/>
-      <c r="E29" s="43"/>
+      <c r="D29" s="55"/>
+      <c r="E29" s="55"/>
       <c r="F29" s="16"/>
       <c r="G29" s="3"/>
       <c r="H29" s="38" t="s">
@@ -1728,19 +1811,17 @@
       <c r="J29" s="3"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B30" s="3" t="s">
+      <c r="A30" s="23"/>
+      <c r="B30" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="C30" s="4">
+      <c r="C30" s="51">
         <v>42947</v>
       </c>
-      <c r="D30" s="21" t="s">
+      <c r="D30" s="58" t="s">
         <v>81</v>
       </c>
-      <c r="E30" s="16">
+      <c r="E30" s="44">
         <v>1</v>
       </c>
       <c r="F30" s="16"/>
@@ -1750,18 +1831,18 @@
       <c r="J30" s="3"/>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A31" s="41"/>
-      <c r="B31" s="41" t="s">
+      <c r="A31" s="23"/>
+      <c r="B31" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="C31" s="42">
+      <c r="C31" s="51">
         <v>42954</v>
       </c>
-      <c r="D31" s="43"/>
-      <c r="E31" s="43"/>
+      <c r="D31" s="44"/>
+      <c r="E31" s="44"/>
       <c r="F31" s="16"/>
       <c r="G31" s="3" t="s">
-        <v>93</v>
+        <v>143</v>
       </c>
       <c r="H31" s="3" t="s">
         <v>133</v>
@@ -1772,19 +1853,19 @@
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A32" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B32" s="3" t="s">
+      <c r="A32" s="53" t="s">
+        <v>37</v>
+      </c>
+      <c r="B32" s="53" t="s">
         <v>44</v>
       </c>
-      <c r="C32" s="4">
+      <c r="C32" s="54">
         <v>42961</v>
       </c>
-      <c r="D32" s="16" t="s">
+      <c r="D32" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="E32" s="16">
+      <c r="E32" s="55">
         <v>1</v>
       </c>
       <c r="F32" s="16"/>
@@ -1796,15 +1877,15 @@
       <c r="J32" s="3"/>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A33" s="41"/>
-      <c r="B33" s="41" t="s">
+      <c r="A33" s="23"/>
+      <c r="B33" s="23" t="s">
         <v>45</v>
       </c>
-      <c r="C33" s="42">
+      <c r="C33" s="51">
         <v>42968</v>
       </c>
-      <c r="D33" s="43"/>
-      <c r="E33" s="43"/>
+      <c r="D33" s="44"/>
+      <c r="E33" s="44"/>
       <c r="F33" s="16"/>
       <c r="G33" s="3"/>
       <c r="H33" s="38" t="s">
@@ -1814,19 +1895,17 @@
       <c r="J33" s="3"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A34" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B34" s="3" t="s">
+      <c r="A34" s="23"/>
+      <c r="B34" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="C34" s="4">
+      <c r="C34" s="51">
         <v>42975</v>
       </c>
-      <c r="D34" s="16" t="s">
+      <c r="D34" s="44" t="s">
         <v>82</v>
       </c>
-      <c r="E34" s="16">
+      <c r="E34" s="44">
         <v>1</v>
       </c>
       <c r="F34" s="16"/>
@@ -1836,20 +1915,22 @@
       <c r="J34" s="3"/>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A35" s="41"/>
-      <c r="B35" s="41" t="s">
+      <c r="A35" s="53" t="s">
+        <v>40</v>
+      </c>
+      <c r="B35" s="53" t="s">
         <v>48</v>
       </c>
-      <c r="C35" s="42">
+      <c r="C35" s="54">
         <v>42982</v>
       </c>
-      <c r="D35" s="43"/>
-      <c r="E35" s="43" t="s">
+      <c r="D35" s="55"/>
+      <c r="E35" s="55" t="s">
         <v>103</v>
       </c>
       <c r="F35" s="16"/>
       <c r="G35" s="3" t="s">
-        <v>94</v>
+        <v>144</v>
       </c>
       <c r="H35" s="3"/>
       <c r="I35" s="3"/>
@@ -1858,19 +1939,17 @@
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A36" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B36" s="3" t="s">
+      <c r="A36" s="23"/>
+      <c r="B36" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="C36" s="4">
+      <c r="C36" s="51">
         <v>42989</v>
       </c>
-      <c r="D36" s="16" t="s">
+      <c r="D36" s="44" t="s">
         <v>82</v>
       </c>
-      <c r="E36" s="16">
+      <c r="E36" s="44">
         <v>1</v>
       </c>
       <c r="F36" s="16"/>
@@ -1882,15 +1961,15 @@
       <c r="J36" s="3"/>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A37" s="41"/>
-      <c r="B37" s="41" t="s">
+      <c r="A37" s="23"/>
+      <c r="B37" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="C37" s="42">
+      <c r="C37" s="51">
         <v>42996</v>
       </c>
-      <c r="D37" s="43"/>
-      <c r="E37" s="43"/>
+      <c r="D37" s="44"/>
+      <c r="E37" s="44"/>
       <c r="F37" s="16"/>
       <c r="G37" s="3"/>
       <c r="H37" s="3" t="s">
@@ -1900,19 +1979,19 @@
       <c r="J37" s="3"/>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A38" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B38" s="3" t="s">
+      <c r="A38" s="53" t="s">
+        <v>43</v>
+      </c>
+      <c r="B38" s="53" t="s">
         <v>53</v>
       </c>
-      <c r="C38" s="4">
+      <c r="C38" s="54">
         <v>43003</v>
       </c>
-      <c r="D38" s="16" t="s">
+      <c r="D38" s="55" t="s">
         <v>87</v>
       </c>
-      <c r="E38" s="16">
+      <c r="E38" s="55">
         <v>1</v>
       </c>
       <c r="F38" s="16"/>
@@ -1924,15 +2003,15 @@
       <c r="J38" s="3"/>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A39" s="41"/>
-      <c r="B39" s="41" t="s">
+      <c r="A39" s="23"/>
+      <c r="B39" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="C39" s="42">
+      <c r="C39" s="51">
         <v>43010</v>
       </c>
-      <c r="D39" s="43"/>
-      <c r="E39" s="43"/>
+      <c r="D39" s="44"/>
+      <c r="E39" s="44"/>
       <c r="F39" s="16"/>
       <c r="G39" s="3"/>
       <c r="H39" s="3"/>
@@ -1942,24 +2021,22 @@
       </c>
     </row>
     <row r="40" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A40" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="B40" s="5" t="s">
+      <c r="A40" s="59"/>
+      <c r="B40" s="59" t="s">
         <v>56</v>
       </c>
-      <c r="C40" s="6">
+      <c r="C40" s="60">
         <v>43017</v>
       </c>
-      <c r="D40" s="5" t="s">
+      <c r="D40" s="59" t="s">
         <v>104</v>
       </c>
-      <c r="E40" s="17">
+      <c r="E40" s="61">
         <v>1</v>
       </c>
       <c r="F40" s="17"/>
       <c r="G40" s="7" t="s">
-        <v>95</v>
+        <v>145</v>
       </c>
       <c r="H40" s="38" t="s">
         <v>135</v>
@@ -1970,15 +2047,17 @@
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A41" s="41"/>
-      <c r="B41" s="41" t="s">
+      <c r="A41" s="53" t="s">
+        <v>46</v>
+      </c>
+      <c r="B41" s="53" t="s">
         <v>58</v>
       </c>
-      <c r="C41" s="42">
+      <c r="C41" s="54">
         <v>43024</v>
       </c>
-      <c r="D41" s="43"/>
-      <c r="E41" s="43"/>
+      <c r="D41" s="55"/>
+      <c r="E41" s="55"/>
       <c r="F41" s="16"/>
       <c r="G41" s="3"/>
       <c r="H41" s="3" t="s">
@@ -1988,19 +2067,17 @@
       <c r="J41" s="3"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A42" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="B42" s="3" t="s">
+      <c r="A42" s="23"/>
+      <c r="B42" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="C42" s="4">
+      <c r="C42" s="51">
         <v>43031</v>
       </c>
-      <c r="D42" s="21" t="s">
+      <c r="D42" s="58" t="s">
         <v>86</v>
       </c>
-      <c r="E42" s="16">
+      <c r="E42" s="44">
         <v>0.8</v>
       </c>
       <c r="F42" s="16"/>
@@ -2014,15 +2091,15 @@
       <c r="J42" s="3"/>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A43" s="3"/>
-      <c r="B43" s="3" t="s">
+      <c r="A43" s="23"/>
+      <c r="B43" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="C43" s="4">
+      <c r="C43" s="51">
         <v>43038</v>
       </c>
-      <c r="D43" s="16"/>
-      <c r="E43" s="16"/>
+      <c r="D43" s="44"/>
+      <c r="E43" s="44"/>
       <c r="F43" s="16"/>
       <c r="G43" s="3"/>
       <c r="H43" s="3"/>
@@ -2034,24 +2111,24 @@
       </c>
     </row>
     <row r="44" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A44" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="B44" s="8" t="s">
+      <c r="A44" s="65" t="s">
+        <v>49</v>
+      </c>
+      <c r="B44" s="62" t="s">
         <v>62</v>
       </c>
-      <c r="C44" s="9">
+      <c r="C44" s="63">
         <v>43045</v>
       </c>
-      <c r="D44" s="8" t="s">
+      <c r="D44" s="62" t="s">
         <v>129</v>
       </c>
-      <c r="E44" s="20">
+      <c r="E44" s="64">
         <v>1</v>
       </c>
       <c r="F44" s="20"/>
       <c r="G44" s="12" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="H44" s="40"/>
       <c r="I44" s="11"/>
@@ -2060,15 +2137,15 @@
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A45" s="3"/>
-      <c r="B45" s="3" t="s">
+      <c r="A45" s="23"/>
+      <c r="B45" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="C45" s="4">
+      <c r="C45" s="51">
         <v>43052</v>
       </c>
-      <c r="D45" s="16"/>
-      <c r="E45" s="16"/>
+      <c r="D45" s="44"/>
+      <c r="E45" s="44"/>
       <c r="F45" s="16"/>
       <c r="G45" s="3"/>
       <c r="H45" s="3" t="s">
@@ -2078,19 +2155,17 @@
       <c r="J45" s="3"/>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A46" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="B46" s="3" t="s">
+      <c r="A46" s="23"/>
+      <c r="B46" s="23" t="s">
         <v>65</v>
       </c>
-      <c r="C46" s="4">
+      <c r="C46" s="51">
         <v>43059</v>
       </c>
-      <c r="D46" s="16" t="s">
+      <c r="D46" s="44" t="s">
         <v>83</v>
       </c>
-      <c r="E46" s="16">
+      <c r="E46" s="44">
         <v>1</v>
       </c>
       <c r="F46" s="16"/>
@@ -2102,15 +2177,17 @@
       <c r="J46" s="3"/>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A47" s="3"/>
-      <c r="B47" s="3" t="s">
+      <c r="A47" s="53" t="s">
+        <v>51</v>
+      </c>
+      <c r="B47" s="53" t="s">
         <v>66</v>
       </c>
-      <c r="C47" s="4">
+      <c r="C47" s="54">
         <v>43066</v>
       </c>
-      <c r="D47" s="16"/>
-      <c r="E47" s="16"/>
+      <c r="D47" s="55"/>
+      <c r="E47" s="55"/>
       <c r="F47" s="16"/>
       <c r="G47" s="3"/>
       <c r="H47" s="38" t="s">
@@ -2120,17 +2197,15 @@
       <c r="J47" s="3"/>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A48" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="B48" s="3" t="s">
+      <c r="A48" s="23"/>
+      <c r="B48" s="23" t="s">
         <v>67</v>
       </c>
-      <c r="C48" s="4">
+      <c r="C48" s="51">
         <v>43073</v>
       </c>
-      <c r="D48" s="16"/>
-      <c r="E48" s="16">
+      <c r="D48" s="44"/>
+      <c r="E48" s="44">
         <v>1</v>
       </c>
       <c r="F48" s="16"/>
@@ -2142,18 +2217,18 @@
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A49" s="3"/>
-      <c r="B49" s="3" t="s">
+      <c r="A49" s="23"/>
+      <c r="B49" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="C49" s="4">
+      <c r="C49" s="51">
         <v>43080</v>
       </c>
-      <c r="D49" s="16"/>
-      <c r="E49" s="16"/>
+      <c r="D49" s="44"/>
+      <c r="E49" s="44"/>
       <c r="F49" s="16"/>
       <c r="G49" s="3" t="s">
-        <v>96</v>
+        <v>147</v>
       </c>
       <c r="H49" s="3"/>
       <c r="I49" s="3"/>
@@ -2189,7 +2264,7 @@
       </c>
       <c r="B52" s="27"/>
       <c r="C52" s="27"/>
-      <c r="D52" s="46" t="s">
+      <c r="D52" s="45" t="s">
         <v>83</v>
       </c>
       <c r="E52" s="28"/>
@@ -2203,7 +2278,7 @@
       <c r="A53" s="30"/>
       <c r="B53" s="23"/>
       <c r="C53" s="23"/>
-      <c r="D53" s="47" t="s">
+      <c r="D53" s="46" t="s">
         <v>129</v>
       </c>
       <c r="E53" s="24"/>
@@ -2217,7 +2292,7 @@
       <c r="A54" s="30"/>
       <c r="B54" s="23"/>
       <c r="C54" s="23"/>
-      <c r="D54" s="47" t="s">
+      <c r="D54" s="46" t="s">
         <v>84</v>
       </c>
       <c r="E54" s="23"/>
@@ -2231,7 +2306,7 @@
       <c r="A55" s="30"/>
       <c r="B55" s="23"/>
       <c r="C55" s="23"/>
-      <c r="D55" s="47" t="s">
+      <c r="D55" s="46" t="s">
         <v>102</v>
       </c>
       <c r="E55" s="23"/>
@@ -2968,7 +3043,7 @@
       <c r="H30" s="3"/>
       <c r="I30" s="3"/>
     </row>
-    <row r="31" spans="1:9" ht="14.45" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
         <v>42</v>
@@ -2987,7 +3062,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="14.45" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>43</v>
       </c>
@@ -3006,7 +3081,7 @@
       <c r="H32" s="3"/>
       <c r="I32" s="3"/>
     </row>
-    <row r="33" spans="1:9" ht="14.45" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="3"/>
       <c r="B33" s="3" t="s">
         <v>45</v>
@@ -3021,7 +3096,7 @@
       <c r="H33" s="3"/>
       <c r="I33" s="3"/>
     </row>
-    <row r="34" spans="1:9" ht="14.45" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>46</v>
       </c>
@@ -3040,7 +3115,7 @@
       <c r="H34" s="3"/>
       <c r="I34" s="3"/>
     </row>
-    <row r="35" spans="1:9" ht="14.45" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="3"/>
       <c r="B35" s="3" t="s">
         <v>48</v>
@@ -3061,7 +3136,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="14.45" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>49</v>
       </c>
@@ -3082,7 +3157,7 @@
       <c r="H36" s="3"/>
       <c r="I36" s="3"/>
     </row>
-    <row r="37" spans="1:9" ht="14.45" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="3"/>
       <c r="B37" s="3" t="s">
         <v>52</v>
@@ -3099,7 +3174,7 @@
       <c r="H37" s="3"/>
       <c r="I37" s="3"/>
     </row>
-    <row r="38" spans="1:9" ht="14.45" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>51</v>
       </c>
@@ -3120,7 +3195,7 @@
       <c r="H38" s="3"/>
       <c r="I38" s="3"/>
     </row>
-    <row r="39" spans="1:9" ht="14.45" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="3"/>
       <c r="B39" s="3" t="s">
         <v>55</v>

</xml_diff>